<commit_message>
Productos alineados con el Vademécum: MP0970 queda como Cliente
La maestra de productos de Visita Comercial ya coincidía con el Vademécum en los 380 productos
generales (nombres y etiquetas). La única diferencia era MP0970 (Vititopic 0.05% Ungüento x 30 g
Envase de Lujo): su Nueva Etiqueta decía Portafolio, pero no está en el portafolio general del
Vademécum. Se deja como Cliente y Portafolio queda en 293, igual que en el Vademécum.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SxueufPeaphr3AnrNJJDTi
</commit_message>
<xml_diff>
--- a/datos/Base_Productos.xlsx
+++ b/datos/Base_Productos.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3268" uniqueCount="1842">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3268" uniqueCount="1843">
   <si>
     <t>Referencia Interna</t>
   </si>
@@ -5567,6 +5567,9 @@
   </si>
   <si>
     <t xml:space="preserve">Este producto es innovador, sugiero revisar envase,cambio de nombre  y hacer lanzamiento </t>
+  </si>
+  <si>
+    <t>Alineado con el Vademécum: no está en el portafolio general, se deja como Cliente</t>
   </si>
 </sst>
 </file>
@@ -15508,10 +15511,10 @@
         <v>34</v>
       </c>
       <c r="F253" s="2" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="G253" s="2" t="s">
-        <v>1830</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="254" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Productos: MP0969 Sedex/Ketodex Emulsión x 30 ml Envase de Lujo pasa a Portafolio
Con la misma categoría de MP0526 (Corticoides / Dermatitis), alineado con el Vademécum.
Las dos apps quedan con los mismos 382 productos generales (Portafolio 295).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SxueufPeaphr3AnrNJJDTi
</commit_message>
<xml_diff>
--- a/datos/Base_Productos.xlsx
+++ b/datos/Base_Productos.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3268" uniqueCount="1842">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3268" uniqueCount="1843">
   <si>
     <t>Referencia Interna</t>
   </si>
@@ -5567,6 +5567,9 @@
   </si>
   <si>
     <t xml:space="preserve">Este producto es innovador, sugiero revisar envase,cambio de nombre  y hacer lanzamiento </t>
+  </si>
+  <si>
+    <t>Producto Epithelium: Portafolio, misma categoría de MP0526</t>
   </si>
 </sst>
 </file>
@@ -15195,7 +15198,7 @@
         <v>1641</v>
       </c>
       <c r="C237" s="2" t="s">
-        <v>615</v>
+        <v>207</v>
       </c>
       <c r="D237" s="2" t="s">
         <v>1637</v>
@@ -15203,8 +15206,12 @@
       <c r="E237" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F237" s="2"/>
-      <c r="G237" s="2"/>
+      <c r="F237" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G237" s="2" t="s">
+        <v>1842</v>
+      </c>
     </row>
     <row r="238" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="2" t="s">

</xml_diff>

<commit_message>
Maestra: enlace Portafolio del cliente con sus productos exclusivos y ficha (componentes, indicación y dosis)
- herramientas/portafolios.py genera portafolios.js: productos con etiqueta Cliente y categoría con el nombre
  del cliente (Base_Productos.xlsx), fichas del Vademécum y cruce con los contactos de la Maestra.
- MP1050 pasa a la categoría Farmapiel Garzón y MP0513 a La Piel del Maestro (como en el Vademécum).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SxueufPeaphr3AnrNJJDTi
</commit_message>
<xml_diff>
--- a/datos/Base_Productos.xlsx
+++ b/datos/Base_Productos.xlsx
@@ -14571,7 +14571,7 @@
         <v>1409</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>51</v>
+        <v>1404</v>
       </c>
       <c r="D204" s="2" t="s">
         <v>1410</v>
@@ -14875,7 +14875,7 @@
         <v>1494</v>
       </c>
       <c r="C220" s="2" t="s">
-        <v>1115</v>
+        <v>55</v>
       </c>
       <c r="D220" s="2" t="s">
         <v>1492</v>

</xml_diff>

<commit_message>
Productos: MP0655 pasa a Med Peeling Forte Crema x 15 g, categoría Tienda Dermocosmética Bella Piel (Cliente)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SxueufPeaphr3AnrNJJDTi
</commit_message>
<xml_diff>
--- a/datos/Base_Productos.xlsx
+++ b/datos/Base_Productos.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3268" uniqueCount="1843">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3269" uniqueCount="1844">
   <si>
     <t>Referencia Interna</t>
   </si>
@@ -5570,6 +5570,9 @@
   </si>
   <si>
     <t>Producto Epithelium: Portafolio, misma categoría de MP0526</t>
+  </si>
+  <si>
+    <t>Med Peeling Forte Crema x 15 g</t>
   </si>
 </sst>
 </file>
@@ -16986,10 +16989,10 @@
         <v>597</v>
       </c>
       <c r="B326" s="2" t="s">
-        <v>598</v>
+        <v>1843</v>
       </c>
       <c r="C326" s="2" t="s">
-        <v>7</v>
+        <v>557</v>
       </c>
       <c r="D326" s="2" t="s">
         <v>599</v>

</xml_diff>